<commit_message>
docs(reports): Consolidado oficial PAS actualizado con 10/19 (v7.4)
</commit_message>
<xml_diff>
--- a/ReportesTrades/PokerDeAses/Tabla_Maestra_PAS.xlsx
+++ b/ReportesTrades/PokerDeAses/Tabla_Maestra_PAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Documents\NinjaTrader 8\bin\Custom\ReportesTrades\PokerDeAses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A3DF0F2-C24D-493A-85D7-4890230EF78B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{608BBCDB-2DFA-45CB-A88E-F19F8FECAB3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29970" yWindow="1200" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{C4916A12-11E2-425A-A1C5-F706448FB038}"/>
+    <workbookView xWindow="29970" yWindow="1200" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{0673FE6F-961A-4C1A-A39C-0275E2529DD7}"/>
   </bookViews>
   <sheets>
     <sheet name="Base_Trades" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="61">
   <si>
     <t>ArchivoOrigen</t>
   </si>
@@ -124,24 +124,60 @@
     <t>Bars</t>
   </si>
   <si>
+    <t>PAS_10192026.xlsx</t>
+  </si>
+  <si>
+    <t>As 2: SOBB</t>
+  </si>
+  <si>
+    <t>ES 12-26</t>
+  </si>
+  <si>
+    <t>Playback101</t>
+  </si>
+  <si>
+    <t>Tick610_PokerDeAsesSniperES</t>
+  </si>
+  <si>
+    <t>Long</t>
+  </si>
+  <si>
+    <t>SOBB_Long</t>
+  </si>
+  <si>
+    <t>SOBB_Tp2_Expansion</t>
+  </si>
+  <si>
+    <t>As 1: Zona 1 (100B)</t>
+  </si>
+  <si>
+    <t>Short</t>
+  </si>
+  <si>
+    <t>Z1-100Bar_Short</t>
+  </si>
+  <si>
+    <t>SL_Midline_Zona1</t>
+  </si>
+  <si>
+    <t>Exit_SOBB_CicloTerminado</t>
+  </si>
+  <si>
+    <t>As 4: Cascada 25</t>
+  </si>
+  <si>
+    <t>Cascada50_Long</t>
+  </si>
+  <si>
+    <t>Cascada_Mono_SL</t>
+  </si>
+  <si>
+    <t>Z1_Mono_Tp</t>
+  </si>
+  <si>
     <t>PAS_10202026.xlsx</t>
   </si>
   <si>
-    <t>As 1: Zona 1 (100B)</t>
-  </si>
-  <si>
-    <t>ES 12-26</t>
-  </si>
-  <si>
-    <t>Playback101</t>
-  </si>
-  <si>
-    <t>Tick610_PokerDeAsesSniperES</t>
-  </si>
-  <si>
-    <t>Long</t>
-  </si>
-  <si>
     <t>Z1-100Bar_Long</t>
   </si>
   <si>
@@ -151,24 +187,6 @@
     <t>Z1_Stop_BE</t>
   </si>
   <si>
-    <t>As 2: SOBB</t>
-  </si>
-  <si>
-    <t>SOBB_Long</t>
-  </si>
-  <si>
-    <t>Exit_SOBB_CicloTerminado</t>
-  </si>
-  <si>
-    <t>As 4: Cascada 25</t>
-  </si>
-  <si>
-    <t>Cascada50_Long</t>
-  </si>
-  <si>
-    <t>Cascada_Mono_SL</t>
-  </si>
-  <si>
     <t>Cascada_Mono_Tp</t>
   </si>
   <si>
@@ -182,15 +200,6 @@
   </si>
   <si>
     <t>Cascada_C3_RunnerAhogo</t>
-  </si>
-  <si>
-    <t>Short</t>
-  </si>
-  <si>
-    <t>Z1-100Bar_Short</t>
-  </si>
-  <si>
-    <t>Z1_Mono_Tp</t>
   </si>
   <si>
     <t>SOBB_Short</t>
@@ -267,8 +276,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -602,8 +611,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C229A281-4D9E-4ADA-837C-6B3F3FE1F712}">
-  <dimension ref="A1:AA16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE66632F-58BA-473C-93F3-20FBB914CD1B}">
+  <dimension ref="A1:AA22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" bestFit="1" customWidth="1"/>
@@ -718,13 +727,13 @@
         <v>27</v>
       </c>
       <c r="B2" s="2">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
       </c>
       <c r="D2">
-        <v>108.14</v>
+        <v>195.64</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -745,16 +754,16 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <v>7732.75</v>
+        <v>7743</v>
       </c>
       <c r="L2">
-        <v>7735</v>
+        <v>7747</v>
       </c>
       <c r="M2" s="3">
-        <v>46315.411527777775</v>
+        <v>46314.425740740742</v>
       </c>
       <c r="N2" s="3">
-        <v>46315.412268518521</v>
+        <v>46314.426435185182</v>
       </c>
       <c r="O2" t="s">
         <v>33</v>
@@ -763,10 +772,10 @@
         <v>34</v>
       </c>
       <c r="Q2" s="4">
-        <v>108.14</v>
+        <v>195.64</v>
       </c>
       <c r="R2" s="4">
-        <v>108.14</v>
+        <v>195.64</v>
       </c>
       <c r="S2" s="4">
         <v>4.3600000000000003</v>
@@ -784,13 +793,13 @@
         <v>0</v>
       </c>
       <c r="X2" s="4">
-        <v>162.5</v>
+        <v>25</v>
       </c>
       <c r="Y2" s="4">
-        <v>112.5</v>
+        <v>275</v>
       </c>
       <c r="Z2" s="4">
-        <v>4.3600000000000003</v>
+        <v>79.36</v>
       </c>
       <c r="AA2">
         <v>9</v>
@@ -801,13 +810,13 @@
         <v>27</v>
       </c>
       <c r="B3" s="2">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D3">
-        <v>216.28</v>
+        <v>-500.58</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -822,37 +831,37 @@
         <v>31</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3">
-        <v>7732.75</v>
+        <v>7742.25</v>
       </c>
       <c r="L3">
-        <v>7735</v>
+        <v>7745.5</v>
       </c>
       <c r="M3" s="3">
-        <v>46315.411527777775</v>
+        <v>46314.441145833334</v>
       </c>
       <c r="N3" s="3">
-        <v>46315.412268518521</v>
+        <v>46314.441736111112</v>
       </c>
       <c r="O3" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="P3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="Q3" s="4">
-        <v>216.28</v>
+        <v>-500.58</v>
       </c>
       <c r="R3" s="4">
-        <v>324.42</v>
+        <v>-304.94</v>
       </c>
       <c r="S3" s="4">
-        <v>8.7200000000000006</v>
+        <v>13.08</v>
       </c>
       <c r="T3" s="4">
         <v>0</v>
@@ -867,16 +876,16 @@
         <v>0</v>
       </c>
       <c r="X3" s="4">
-        <v>325</v>
+        <v>525</v>
       </c>
       <c r="Y3" s="4">
-        <v>225</v>
+        <v>112.5</v>
       </c>
       <c r="Z3" s="4">
-        <v>8.7200000000000006</v>
+        <v>613.08000000000004</v>
       </c>
       <c r="AA3">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
@@ -884,13 +893,13 @@
         <v>27</v>
       </c>
       <c r="B4" s="2">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D4">
-        <v>58.14</v>
+        <v>70.64</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -911,28 +920,28 @@
         <v>1</v>
       </c>
       <c r="K4">
-        <v>7736.5</v>
+        <v>7754.5</v>
       </c>
       <c r="L4">
-        <v>7737.75</v>
+        <v>7756</v>
       </c>
       <c r="M4" s="3">
-        <v>46315.412326388891</v>
+        <v>46314.458599537036</v>
       </c>
       <c r="N4" s="3">
-        <v>46315.414224537039</v>
+        <v>46314.462754629632</v>
       </c>
       <c r="O4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="P4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q4" s="4">
-        <v>58.14</v>
+        <v>70.64</v>
       </c>
       <c r="R4" s="4">
-        <v>382.56</v>
+        <v>-234.3</v>
       </c>
       <c r="S4" s="4">
         <v>4.3600000000000003</v>
@@ -950,16 +959,16 @@
         <v>0</v>
       </c>
       <c r="X4" s="4">
-        <v>212.5</v>
+        <v>237.5</v>
       </c>
       <c r="Y4" s="4">
         <v>175</v>
       </c>
       <c r="Z4" s="4">
-        <v>116.86</v>
+        <v>104.36</v>
       </c>
       <c r="AA4">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
@@ -967,13 +976,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="2">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D5">
-        <v>-204.36</v>
+        <v>-116.86</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -994,28 +1003,28 @@
         <v>1</v>
       </c>
       <c r="K5">
-        <v>7751.75</v>
+        <v>7770.75</v>
       </c>
       <c r="L5">
-        <v>7747.75</v>
+        <v>7768.5</v>
       </c>
       <c r="M5" s="3">
-        <v>46315.41847222222</v>
+        <v>46314.477847222224</v>
       </c>
       <c r="N5" s="3">
-        <v>46315.418773148151</v>
+        <v>46314.478819444441</v>
       </c>
       <c r="O5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q5" s="4">
-        <v>-204.36</v>
+        <v>-116.86</v>
       </c>
       <c r="R5" s="4">
-        <v>178.2</v>
+        <v>-351.16</v>
       </c>
       <c r="S5" s="4">
         <v>4.3600000000000003</v>
@@ -1033,16 +1042,16 @@
         <v>0</v>
       </c>
       <c r="X5" s="4">
-        <v>200</v>
+        <v>162.5</v>
       </c>
       <c r="Y5" s="4">
-        <v>12.5</v>
+        <v>25</v>
       </c>
       <c r="Z5" s="4">
-        <v>216.86</v>
+        <v>141.86000000000001</v>
       </c>
       <c r="AA5">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
@@ -1050,13 +1059,13 @@
         <v>27</v>
       </c>
       <c r="B6" s="2">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D6">
-        <v>170.64</v>
+        <v>-179.36</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -1077,28 +1086,28 @@
         <v>1</v>
       </c>
       <c r="K6">
-        <v>7752.25</v>
+        <v>7771.75</v>
       </c>
       <c r="L6">
-        <v>7755.75</v>
+        <v>7768.25</v>
       </c>
       <c r="M6" s="3">
-        <v>46315.421759259261</v>
+        <v>46314.483831018515</v>
       </c>
       <c r="N6" s="3">
-        <v>46315.421944444446</v>
+        <v>46314.486250000002</v>
       </c>
       <c r="O6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P6" t="s">
         <v>42</v>
       </c>
       <c r="Q6" s="4">
-        <v>170.64</v>
+        <v>-179.36</v>
       </c>
       <c r="R6" s="4">
-        <v>348.84</v>
+        <v>-530.52</v>
       </c>
       <c r="S6" s="4">
         <v>4.3600000000000003</v>
@@ -1116,16 +1125,16 @@
         <v>0</v>
       </c>
       <c r="X6" s="4">
-        <v>12.5</v>
+        <v>175</v>
       </c>
       <c r="Y6" s="4">
-        <v>175</v>
+        <v>75</v>
       </c>
       <c r="Z6" s="4">
-        <v>4.3600000000000003</v>
+        <v>254.36</v>
       </c>
       <c r="AA6">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
@@ -1133,13 +1142,13 @@
         <v>27</v>
       </c>
       <c r="B7" s="2">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D7">
-        <v>8.14</v>
+        <v>95.64</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -1154,34 +1163,34 @@
         <v>31</v>
       </c>
       <c r="I7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7">
-        <v>7755.75</v>
+        <v>7751.25</v>
       </c>
       <c r="L7">
-        <v>7756</v>
+        <v>7749.25</v>
       </c>
       <c r="M7" s="3">
-        <v>46315.424467592595</v>
+        <v>46314.50273148148</v>
       </c>
       <c r="N7" s="3">
-        <v>46315.426168981481</v>
+        <v>46314.504490740743</v>
       </c>
       <c r="O7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="P7" t="s">
         <v>43</v>
       </c>
       <c r="Q7" s="4">
-        <v>8.14</v>
+        <v>95.64</v>
       </c>
       <c r="R7" s="4">
-        <v>356.98</v>
+        <v>-434.88</v>
       </c>
       <c r="S7" s="4">
         <v>4.3600000000000003</v>
@@ -1199,33 +1208,33 @@
         <v>0</v>
       </c>
       <c r="X7" s="4">
-        <v>137.5</v>
+        <v>162.5</v>
       </c>
       <c r="Y7" s="4">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="Z7" s="4">
-        <v>91.86</v>
+        <v>54.36</v>
       </c>
       <c r="AA7">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B8" s="2">
         <v>46315</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D8">
-        <v>16.28</v>
+        <v>108.14</v>
       </c>
       <c r="E8">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F8" t="s">
         <v>29</v>
@@ -1240,34 +1249,34 @@
         <v>32</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>7755.75</v>
+        <v>7732.75</v>
       </c>
       <c r="L8">
-        <v>7756</v>
+        <v>7735</v>
       </c>
       <c r="M8" s="3">
-        <v>46315.424467592595</v>
+        <v>46315.411527777775</v>
       </c>
       <c r="N8" s="3">
-        <v>46315.426168981481</v>
+        <v>46315.412268518521</v>
       </c>
       <c r="O8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="P8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Q8" s="4">
-        <v>16.28</v>
+        <v>108.14</v>
       </c>
       <c r="R8" s="4">
-        <v>373.26</v>
+        <v>108.14</v>
       </c>
       <c r="S8" s="4">
-        <v>8.7200000000000006</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="T8" s="4">
         <v>0</v>
@@ -1282,33 +1291,33 @@
         <v>0</v>
       </c>
       <c r="X8" s="4">
-        <v>275</v>
+        <v>162.5</v>
       </c>
       <c r="Y8" s="4">
-        <v>200</v>
+        <v>112.5</v>
       </c>
       <c r="Z8" s="4">
-        <v>183.72</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="AA8">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B9" s="2">
         <v>46315</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D9">
-        <v>120.64</v>
+        <v>216.28</v>
       </c>
       <c r="E9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -1323,34 +1332,34 @@
         <v>32</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9">
-        <v>7763.75</v>
+        <v>7732.75</v>
       </c>
       <c r="L9">
-        <v>7766.25</v>
+        <v>7735</v>
       </c>
       <c r="M9" s="3">
-        <v>46315.429027777776</v>
+        <v>46315.411527777775</v>
       </c>
       <c r="N9" s="3">
-        <v>46315.429895833331</v>
+        <v>46315.412268518521</v>
       </c>
       <c r="O9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="P9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q9" s="4">
-        <v>120.64</v>
+        <v>216.28</v>
       </c>
       <c r="R9" s="4">
-        <v>493.9</v>
+        <v>324.42</v>
       </c>
       <c r="S9" s="4">
-        <v>4.3600000000000003</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="T9" s="4">
         <v>0</v>
@@ -1365,13 +1374,13 @@
         <v>0</v>
       </c>
       <c r="X9" s="4">
-        <v>37.5</v>
+        <v>325</v>
       </c>
       <c r="Y9" s="4">
-        <v>212.5</v>
+        <v>225</v>
       </c>
       <c r="Z9" s="4">
-        <v>91.86</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="AA9">
         <v>9</v>
@@ -1379,19 +1388,19 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B10" s="2">
         <v>46315</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D10">
-        <v>170.64</v>
+        <v>58.14</v>
       </c>
       <c r="E10">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -1409,28 +1418,28 @@
         <v>1</v>
       </c>
       <c r="K10">
-        <v>7763.75</v>
+        <v>7736.5</v>
       </c>
       <c r="L10">
-        <v>7767.25</v>
+        <v>7737.75</v>
       </c>
       <c r="M10" s="3">
-        <v>46315.429027777776</v>
+        <v>46315.412326388891</v>
       </c>
       <c r="N10" s="3">
-        <v>46315.430219907408</v>
+        <v>46315.414224537039</v>
       </c>
       <c r="O10" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="P10" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="Q10" s="4">
-        <v>170.64</v>
+        <v>58.14</v>
       </c>
       <c r="R10" s="4">
-        <v>664.54</v>
+        <v>382.56</v>
       </c>
       <c r="S10" s="4">
         <v>4.3600000000000003</v>
@@ -1448,33 +1457,33 @@
         <v>0</v>
       </c>
       <c r="X10" s="4">
-        <v>37.5</v>
+        <v>212.5</v>
       </c>
       <c r="Y10" s="4">
-        <v>212.5</v>
+        <v>175</v>
       </c>
       <c r="Z10" s="4">
-        <v>41.86</v>
+        <v>116.86</v>
       </c>
       <c r="AA10">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B11" s="2">
         <v>46315</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11">
-        <v>120.64</v>
+        <v>-204.36</v>
       </c>
       <c r="E11">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -1492,28 +1501,28 @@
         <v>1</v>
       </c>
       <c r="K11">
-        <v>7763.75</v>
+        <v>7751.75</v>
       </c>
       <c r="L11">
-        <v>7766.25</v>
+        <v>7747.75</v>
       </c>
       <c r="M11" s="3">
-        <v>46315.429027777776</v>
+        <v>46315.41847222222</v>
       </c>
       <c r="N11" s="3">
-        <v>46315.430555555555</v>
+        <v>46315.418773148151</v>
       </c>
       <c r="O11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q11" s="4">
-        <v>120.64</v>
+        <v>-204.36</v>
       </c>
       <c r="R11" s="4">
-        <v>785.18</v>
+        <v>178.2</v>
       </c>
       <c r="S11" s="4">
         <v>4.3600000000000003</v>
@@ -1531,33 +1540,33 @@
         <v>0</v>
       </c>
       <c r="X11" s="4">
-        <v>37.5</v>
+        <v>200</v>
       </c>
       <c r="Y11" s="4">
-        <v>212.5</v>
+        <v>12.5</v>
       </c>
       <c r="Z11" s="4">
-        <v>91.86</v>
+        <v>216.86</v>
       </c>
       <c r="AA11">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B12" s="2">
         <v>46315</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D12">
-        <v>95.64</v>
+        <v>170.64</v>
       </c>
       <c r="E12">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
@@ -1575,28 +1584,28 @@
         <v>1</v>
       </c>
       <c r="K12">
-        <v>7771.5</v>
+        <v>7752.25</v>
       </c>
       <c r="L12">
-        <v>7773.5</v>
+        <v>7755.75</v>
       </c>
       <c r="M12" s="3">
-        <v>46315.433298611111</v>
+        <v>46315.421759259261</v>
       </c>
       <c r="N12" s="3">
-        <v>46315.433553240742</v>
+        <v>46315.421944444446</v>
       </c>
       <c r="O12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P12" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="Q12" s="4">
-        <v>95.64</v>
+        <v>170.64</v>
       </c>
       <c r="R12" s="4">
-        <v>880.82</v>
+        <v>348.84</v>
       </c>
       <c r="S12" s="4">
         <v>4.3600000000000003</v>
@@ -1614,33 +1623,33 @@
         <v>0</v>
       </c>
       <c r="X12" s="4">
-        <v>75</v>
+        <v>12.5</v>
       </c>
       <c r="Y12" s="4">
-        <v>112.5</v>
+        <v>175</v>
       </c>
       <c r="Z12" s="4">
-        <v>16.86</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="AA12">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B13" s="2">
         <v>46315</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13">
-        <v>166.28</v>
+        <v>8.14</v>
       </c>
       <c r="E13">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -1655,34 +1664,34 @@
         <v>32</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13">
-        <v>7775.75</v>
+        <v>7755.75</v>
       </c>
       <c r="L13">
-        <v>7777.5</v>
+        <v>7756</v>
       </c>
       <c r="M13" s="3">
-        <v>46315.435578703706</v>
+        <v>46315.424467592595</v>
       </c>
       <c r="N13" s="3">
-        <v>46315.435624999998</v>
+        <v>46315.426168981481</v>
       </c>
       <c r="O13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P13" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="Q13" s="4">
-        <v>166.28</v>
+        <v>8.14</v>
       </c>
       <c r="R13" s="4">
-        <v>1047.0999999999999</v>
+        <v>356.98</v>
       </c>
       <c r="S13" s="4">
-        <v>8.7200000000000006</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="T13" s="4">
         <v>0</v>
@@ -1697,33 +1706,33 @@
         <v>0</v>
       </c>
       <c r="X13" s="4">
-        <v>25</v>
+        <v>137.5</v>
       </c>
       <c r="Y13" s="4">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="Z13" s="4">
-        <v>33.72</v>
+        <v>91.86</v>
       </c>
       <c r="AA13">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2">
         <v>46315</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D14">
-        <v>45.64</v>
+        <v>16.28</v>
       </c>
       <c r="E14">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F14" t="s">
         <v>29</v>
@@ -1738,34 +1747,34 @@
         <v>32</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14">
-        <v>7785.5</v>
+        <v>7755.75</v>
       </c>
       <c r="L14">
-        <v>7786.5</v>
+        <v>7756</v>
       </c>
       <c r="M14" s="3">
-        <v>46315.437557870369</v>
+        <v>46315.424467592595</v>
       </c>
       <c r="N14" s="3">
-        <v>46315.437696759262</v>
+        <v>46315.426168981481</v>
       </c>
       <c r="O14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P14" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="Q14" s="4">
-        <v>45.64</v>
+        <v>16.28</v>
       </c>
       <c r="R14" s="4">
-        <v>1092.74</v>
+        <v>373.26</v>
       </c>
       <c r="S14" s="4">
-        <v>4.3600000000000003</v>
+        <v>8.7200000000000006</v>
       </c>
       <c r="T14" s="4">
         <v>0</v>
@@ -1780,33 +1789,33 @@
         <v>0</v>
       </c>
       <c r="X14" s="4">
-        <v>25</v>
+        <v>275</v>
       </c>
       <c r="Y14" s="4">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="Z14" s="4">
-        <v>54.36</v>
+        <v>183.72</v>
       </c>
       <c r="AA14">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B15" s="2">
         <v>46315</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D15">
         <v>120.64</v>
       </c>
       <c r="E15">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
@@ -1818,25 +1827,25 @@
         <v>31</v>
       </c>
       <c r="I15" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="J15">
         <v>1</v>
       </c>
       <c r="K15">
-        <v>7776.75</v>
+        <v>7763.75</v>
       </c>
       <c r="L15">
-        <v>7774.25</v>
+        <v>7766.25</v>
       </c>
       <c r="M15" s="3">
-        <v>46315.465763888889</v>
+        <v>46315.429027777776</v>
       </c>
       <c r="N15" s="3">
-        <v>46315.466180555559</v>
+        <v>46315.429895833331</v>
       </c>
       <c r="O15" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="P15" t="s">
         <v>49</v>
@@ -1845,7 +1854,7 @@
         <v>120.64</v>
       </c>
       <c r="R15" s="4">
-        <v>1213.3800000000001</v>
+        <v>493.9</v>
       </c>
       <c r="S15" s="4">
         <v>4.3600000000000003</v>
@@ -1863,33 +1872,33 @@
         <v>0</v>
       </c>
       <c r="X15" s="4">
-        <v>25</v>
+        <v>37.5</v>
       </c>
       <c r="Y15" s="4">
-        <v>150</v>
+        <v>212.5</v>
       </c>
       <c r="Z15" s="4">
-        <v>29.36</v>
+        <v>91.86</v>
       </c>
       <c r="AA15">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="B16" s="2">
         <v>46315</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D16">
-        <v>-129.36000000000001</v>
+        <v>170.64</v>
       </c>
       <c r="E16">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F16" t="s">
         <v>29</v>
@@ -1901,34 +1910,34 @@
         <v>31</v>
       </c>
       <c r="I16" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="J16">
         <v>1</v>
       </c>
       <c r="K16">
-        <v>7772.5</v>
+        <v>7763.75</v>
       </c>
       <c r="L16">
-        <v>7775</v>
+        <v>7767.25</v>
       </c>
       <c r="M16" s="3">
-        <v>46315.466284722221</v>
+        <v>46315.429027777776</v>
       </c>
       <c r="N16" s="3">
-        <v>46315.466620370367</v>
+        <v>46315.430219907408</v>
       </c>
       <c r="O16" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="P16" t="s">
         <v>51</v>
       </c>
       <c r="Q16" s="4">
-        <v>-129.36000000000001</v>
+        <v>170.64</v>
       </c>
       <c r="R16" s="4">
-        <v>1084.02</v>
+        <v>664.54</v>
       </c>
       <c r="S16" s="4">
         <v>4.3600000000000003</v>
@@ -1946,15 +1955,513 @@
         <v>0</v>
       </c>
       <c r="X16" s="4">
+        <v>37.5</v>
+      </c>
+      <c r="Y16" s="4">
+        <v>212.5</v>
+      </c>
+      <c r="Z16" s="4">
+        <v>41.86</v>
+      </c>
+      <c r="AA16">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17">
+        <v>120.64</v>
+      </c>
+      <c r="E17">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17" t="s">
+        <v>32</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>7763.75</v>
+      </c>
+      <c r="L17">
+        <v>7766.25</v>
+      </c>
+      <c r="M17" s="3">
+        <v>46315.429027777776</v>
+      </c>
+      <c r="N17" s="3">
+        <v>46315.430555555555</v>
+      </c>
+      <c r="O17" t="s">
+        <v>41</v>
+      </c>
+      <c r="P17" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q17" s="4">
+        <v>120.64</v>
+      </c>
+      <c r="R17" s="4">
+        <v>785.18</v>
+      </c>
+      <c r="S17" s="4">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="T17" s="4">
+        <v>0</v>
+      </c>
+      <c r="U17" s="4">
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
+        <v>0</v>
+      </c>
+      <c r="W17" s="4">
+        <v>0</v>
+      </c>
+      <c r="X17" s="4">
+        <v>37.5</v>
+      </c>
+      <c r="Y17" s="4">
+        <v>212.5</v>
+      </c>
+      <c r="Z17" s="4">
+        <v>91.86</v>
+      </c>
+      <c r="AA17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18">
+        <v>95.64</v>
+      </c>
+      <c r="E18">
+        <v>11</v>
+      </c>
+      <c r="F18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" t="s">
+        <v>31</v>
+      </c>
+      <c r="I18" t="s">
+        <v>32</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <v>7771.5</v>
+      </c>
+      <c r="L18">
+        <v>7773.5</v>
+      </c>
+      <c r="M18" s="3">
+        <v>46315.433298611111</v>
+      </c>
+      <c r="N18" s="3">
+        <v>46315.433553240742</v>
+      </c>
+      <c r="O18" t="s">
+        <v>41</v>
+      </c>
+      <c r="P18" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q18" s="4">
+        <v>95.64</v>
+      </c>
+      <c r="R18" s="4">
+        <v>880.82</v>
+      </c>
+      <c r="S18" s="4">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="T18" s="4">
+        <v>0</v>
+      </c>
+      <c r="U18" s="4">
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
+        <v>0</v>
+      </c>
+      <c r="W18" s="4">
+        <v>0</v>
+      </c>
+      <c r="X18" s="4">
+        <v>75</v>
+      </c>
+      <c r="Y18" s="4">
+        <v>112.5</v>
+      </c>
+      <c r="Z18" s="4">
+        <v>16.86</v>
+      </c>
+      <c r="AA18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19">
+        <v>166.28</v>
+      </c>
+      <c r="E19">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" t="s">
+        <v>31</v>
+      </c>
+      <c r="I19" t="s">
+        <v>32</v>
+      </c>
+      <c r="J19">
+        <v>2</v>
+      </c>
+      <c r="K19">
+        <v>7775.75</v>
+      </c>
+      <c r="L19">
+        <v>7777.5</v>
+      </c>
+      <c r="M19" s="3">
+        <v>46315.435578703706</v>
+      </c>
+      <c r="N19" s="3">
+        <v>46315.435624999998</v>
+      </c>
+      <c r="O19" t="s">
+        <v>41</v>
+      </c>
+      <c r="P19" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q19" s="4">
+        <v>166.28</v>
+      </c>
+      <c r="R19" s="4">
+        <v>1047.0999999999999</v>
+      </c>
+      <c r="S19" s="4">
+        <v>8.7200000000000006</v>
+      </c>
+      <c r="T19" s="4">
+        <v>0</v>
+      </c>
+      <c r="U19" s="4">
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
+        <v>0</v>
+      </c>
+      <c r="W19" s="4">
+        <v>0</v>
+      </c>
+      <c r="X19" s="4">
+        <v>25</v>
+      </c>
+      <c r="Y19" s="4">
+        <v>200</v>
+      </c>
+      <c r="Z19" s="4">
+        <v>33.72</v>
+      </c>
+      <c r="AA19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C20" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20">
+        <v>45.64</v>
+      </c>
+      <c r="E20">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
+        <v>29</v>
+      </c>
+      <c r="G20" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" t="s">
+        <v>32</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+      <c r="K20">
+        <v>7785.5</v>
+      </c>
+      <c r="L20">
+        <v>7786.5</v>
+      </c>
+      <c r="M20" s="3">
+        <v>46315.437557870369</v>
+      </c>
+      <c r="N20" s="3">
+        <v>46315.437696759262</v>
+      </c>
+      <c r="O20" t="s">
+        <v>41</v>
+      </c>
+      <c r="P20" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q20" s="4">
+        <v>45.64</v>
+      </c>
+      <c r="R20" s="4">
+        <v>1092.74</v>
+      </c>
+      <c r="S20" s="4">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="T20" s="4">
+        <v>0</v>
+      </c>
+      <c r="U20" s="4">
+        <v>0</v>
+      </c>
+      <c r="V20" s="4">
+        <v>0</v>
+      </c>
+      <c r="W20" s="4">
+        <v>0</v>
+      </c>
+      <c r="X20" s="4">
+        <v>25</v>
+      </c>
+      <c r="Y20" s="4">
+        <v>100</v>
+      </c>
+      <c r="Z20" s="4">
+        <v>54.36</v>
+      </c>
+      <c r="AA20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21">
+        <v>120.64</v>
+      </c>
+      <c r="E21">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>29</v>
+      </c>
+      <c r="G21" t="s">
+        <v>30</v>
+      </c>
+      <c r="H21" t="s">
+        <v>31</v>
+      </c>
+      <c r="I21" t="s">
+        <v>36</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>7776.75</v>
+      </c>
+      <c r="L21">
+        <v>7774.25</v>
+      </c>
+      <c r="M21" s="3">
+        <v>46315.465763888889</v>
+      </c>
+      <c r="N21" s="3">
+        <v>46315.466180555559</v>
+      </c>
+      <c r="O21" t="s">
+        <v>37</v>
+      </c>
+      <c r="P21" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q21" s="4">
+        <v>120.64</v>
+      </c>
+      <c r="R21" s="4">
+        <v>1213.3800000000001</v>
+      </c>
+      <c r="S21" s="4">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="T21" s="4">
+        <v>0</v>
+      </c>
+      <c r="U21" s="4">
+        <v>0</v>
+      </c>
+      <c r="V21" s="4">
+        <v>0</v>
+      </c>
+      <c r="W21" s="4">
+        <v>0</v>
+      </c>
+      <c r="X21" s="4">
+        <v>25</v>
+      </c>
+      <c r="Y21" s="4">
         <v>150</v>
       </c>
-      <c r="Y16" s="4">
+      <c r="Z21" s="4">
+        <v>29.36</v>
+      </c>
+      <c r="AA21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="2">
+        <v>46315</v>
+      </c>
+      <c r="C22" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22">
+        <v>-129.36000000000001</v>
+      </c>
+      <c r="E22">
+        <v>15</v>
+      </c>
+      <c r="F22" t="s">
+        <v>29</v>
+      </c>
+      <c r="G22" t="s">
+        <v>30</v>
+      </c>
+      <c r="H22" t="s">
+        <v>31</v>
+      </c>
+      <c r="I22" t="s">
+        <v>36</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <v>7772.5</v>
+      </c>
+      <c r="L22">
+        <v>7775</v>
+      </c>
+      <c r="M22" s="3">
+        <v>46315.466284722221</v>
+      </c>
+      <c r="N22" s="3">
+        <v>46315.466620370367</v>
+      </c>
+      <c r="O22" t="s">
+        <v>53</v>
+      </c>
+      <c r="P22" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q22" s="4">
+        <v>-129.36000000000001</v>
+      </c>
+      <c r="R22" s="4">
+        <v>1084.02</v>
+      </c>
+      <c r="S22" s="4">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="T22" s="4">
+        <v>0</v>
+      </c>
+      <c r="U22" s="4">
+        <v>0</v>
+      </c>
+      <c r="V22" s="4">
+        <v>0</v>
+      </c>
+      <c r="W22" s="4">
+        <v>0</v>
+      </c>
+      <c r="X22" s="4">
+        <v>150</v>
+      </c>
+      <c r="Y22" s="4">
         <v>12.5</v>
       </c>
-      <c r="Z16" s="4">
+      <c r="Z22" s="4">
         <v>141.86000000000001</v>
       </c>
-      <c r="AA16">
+      <c r="AA22">
         <v>4</v>
       </c>
     </row>
@@ -1964,8 +2471,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B556CB6B-EEDE-4EC0-A07F-D9CC00AEDEDF}">
-  <dimension ref="A1:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B00CC1C0-7BB1-49A9-B92D-6C98178B6AD7}">
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1981,38 +2488,58 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
+        <v>46314</v>
+      </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F2">
+        <v>-434.88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>46315</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>15</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>13</v>
       </c>
-      <c r="D2">
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E3" s="6">
         <v>0.86699999999999999</v>
       </c>
-      <c r="F2">
+      <c r="F3">
         <v>1084.02</v>
       </c>
     </row>
@@ -2022,7 +2549,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7737D0E8-5AEB-4E8F-9C06-1BF5203D5486}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B42B401-70DA-441A-AF3C-B0A79E83B58E}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2036,22 +2563,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2059,50 +2586,53 @@
         <v>28</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>1</v>
+      <c r="E2" s="5">
+        <v>0.75</v>
       </c>
       <c r="F2">
-        <v>445.06</v>
+        <v>195.06</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="E3" s="6">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.8</v>
       </c>
       <c r="F3">
-        <v>-71.22</v>
+        <v>40.119999999999997</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4">
         <v>9</v>
       </c>
-      <c r="E4" s="6">
-        <v>0.9</v>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.75</v>
       </c>
       <c r="F4">
-        <v>710.18</v>
+        <v>413.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>